<commit_message>
Add project implementations, prompts, eval scripts and gitignore
- Add src implementations for projects 1-7 (main.py, README, requirements, etc.)
- Add prompt.md files for projects 1-50
- Add run_eval.py with timeout handling and file comparison support
- Add batch_test.py, test_single.py, test_with_judge.py
- Add .gitignore for __pycache__, .pyc, .db, test_results.json
- Fix eval timeout issue for interactive shell tests
- Fix file_comparison test to handle non-README comparisons

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRDBench/6/evaluation/split_output.xlsx
+++ b/PRDBench/6/evaluation/split_output.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="华东" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="华北" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="华南" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="华北" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="华南" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="华东" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,11 +445,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>华东</t>
+          <t>华北</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>300</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>华北</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -481,21 +491,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>华北</t>
+          <t>华南</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>华北</t>
+          <t>华南</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -509,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,21 +537,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>华南</t>
+          <t>华东</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>华南</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>